<commit_message>
v2.0.0: ILAW tab runs on the built-in BOW library — Grade → Subject → Topic dropdowns
- Scan the Desktop "DepEd BOW Files" library once (13 grade folders, 241 subjects,
  289 PDFs) and cache it on disk, so teachers pick a lesson instead of uploading a BOW.
- Topic dropdown shows "Term · Week — Lesson" straight from the BOW; no-term SHS
  Grade 11/12 BOWs show "Week N — topic", SHS units and Kindergarten themes show the title.
- The AI now decides the session count (SCHEMA session_count, clamped 1–5): the
  teacher no longer picks it.
- Learning Area, Term, and Lesson title lock from the selected topic; manual BOW
  upload stays as a fallback expander.
- parse_bow accepts week rows without term headings; new extractors cover SHS units
  (before/after-competency + Roman-numeral), Tech-Pro single-week rows, and Kinder themes.
- 20/20 test suites pass; installer rebuilt; README Tab 1 rewritten.

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/SAMPLE ILAW FORMAT_WIDE.xlsx
+++ b/SAMPLE ILAW FORMAT_WIDE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Documents\Codex\2026-09-18\i\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD8B3AAF-0083-455E-9AE4-7DEA908A7F09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A521E08-9069-4CD1-9DB2-B3A14412859F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -141,9 +141,6 @@
   </si>
   <si>
     <t>Name of Teacher</t>
-  </si>
-  <si>
-    <t>Week</t>
   </si>
   <si>
     <t>Week 3</t>
@@ -374,6 +371,9 @@
   </si>
   <si>
     <t>NAME OF MASTER TEACHER</t>
+  </si>
+  <si>
+    <t>Term/Week</t>
   </si>
 </sst>
 </file>
@@ -587,71 +587,71 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -979,146 +979,146 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
+      <c r="B5" s="18"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
     </row>
     <row r="7" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
     </row>
     <row r="8" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="20" t="s">
-        <v>44</v>
-      </c>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="19"/>
+      <c r="B8" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="16"/>
     </row>
     <row r="9" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="19"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="16"/>
     </row>
     <row r="10" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="19"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="16"/>
     </row>
     <row r="11" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="17" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="19"/>
+      <c r="B11" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="16"/>
     </row>
     <row r="12" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B12" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="19"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="16"/>
     </row>
     <row r="13" spans="1:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B13" s="30">
+        <v>40</v>
+      </c>
+      <c r="B13" s="27">
         <v>5</v>
       </c>
-      <c r="C13" s="31"/>
-      <c r="D13" s="31"/>
-      <c r="E13" s="31"/>
-      <c r="F13" s="20"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="29"/>
     </row>
     <row r="14" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
@@ -1142,68 +1142,68 @@
     </row>
     <row r="15" spans="1:6" ht="93" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="B15" s="25" t="s">
-        <v>46</v>
-      </c>
-      <c r="C15" s="26"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="26"/>
-      <c r="F15" s="27"/>
+        <v>81</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="C15" s="23"/>
+      <c r="D15" s="23"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="24"/>
     </row>
     <row r="16" spans="1:6" ht="98.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B16" s="25" t="s">
-        <v>42</v>
-      </c>
-      <c r="C16" s="28"/>
-      <c r="D16" s="28"/>
-      <c r="E16" s="28"/>
-      <c r="F16" s="29"/>
+        <v>82</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" s="25"/>
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="26"/>
     </row>
     <row r="17" spans="1:6" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="15"/>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="16"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="13"/>
     </row>
     <row r="18" spans="1:6" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="32" t="s">
-        <v>45</v>
-      </c>
-      <c r="C18" s="33"/>
-      <c r="D18" s="33"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="34"/>
+      <c r="B18" s="30" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="32"/>
     </row>
     <row r="19" spans="1:6" ht="106.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B19" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="C19" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="D19" s="9" t="s">
+      <c r="E19" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="E19" s="9" t="s">
-        <v>49</v>
-      </c>
       <c r="F19" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
@@ -1217,153 +1217,153 @@
       <c r="F20" s="37"/>
     </row>
     <row r="21" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="15"/>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="16"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="13"/>
     </row>
     <row r="22" spans="1:6" ht="111.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B22" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C22" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="D22" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="E22" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="E22" s="9" t="s">
-        <v>53</v>
-      </c>
       <c r="F22" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="180.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B23" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C23" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="D23" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="E23" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E23" s="9" t="s">
+      <c r="F23" s="9" t="s">
         <v>57</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="36" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B24" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C24" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="D24" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="E24" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="E24" s="9" t="s">
-        <v>62</v>
-      </c>
       <c r="F24" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="48" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B25" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="C25" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="D25" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="E25" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="E25" s="9" t="s">
-        <v>66</v>
-      </c>
       <c r="F25" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="14" t="s">
+      <c r="A26" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B26" s="15"/>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="15"/>
-      <c r="F26" s="16"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="13"/>
     </row>
     <row r="27" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B27" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="C27" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="D27" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="E27" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="F27" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="F27" s="9" t="s">
-        <v>71</v>
-      </c>
     </row>
     <row r="28" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="14" t="s">
+      <c r="A28" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="15"/>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="15"/>
-      <c r="F28" s="16"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="13"/>
     </row>
     <row r="29" spans="1:6" ht="48" x14ac:dyDescent="0.3">
       <c r="A29" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B29" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C29" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="D29" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="D29" s="9" t="s">
+      <c r="E29" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="E29" s="9" t="s">
-        <v>75</v>
-      </c>
       <c r="F29" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="48" x14ac:dyDescent="0.3">
@@ -1395,77 +1395,59 @@
       <c r="F31" s="6"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="24" t="s">
+      <c r="A32" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B32" s="12"/>
-      <c r="C32" s="24" t="s">
+      <c r="B32" s="18"/>
+      <c r="C32" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="D32" s="12"/>
-      <c r="E32" s="24" t="s">
+      <c r="D32" s="18"/>
+      <c r="E32" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="F32" s="12"/>
+      <c r="F32" s="18"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="22" t="s">
+      <c r="A34" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="B34" s="12"/>
-      <c r="C34" s="22" t="s">
-        <v>85</v>
-      </c>
-      <c r="D34" s="12"/>
-      <c r="E34" s="22" t="s">
+      <c r="B34" s="18"/>
+      <c r="C34" s="19" t="s">
         <v>84</v>
       </c>
-      <c r="F34" s="12"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="F34" s="18"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="21" t="s">
+      <c r="A35" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="B35" s="12"/>
-      <c r="C35" s="21" t="s">
+      <c r="B35" s="18"/>
+      <c r="C35" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D35" s="12"/>
-      <c r="E35" s="21" t="s">
+      <c r="D35" s="18"/>
+      <c r="E35" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="F35" s="12"/>
+      <c r="F35" s="18"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="23" t="s">
+      <c r="A38" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="B38" s="12"/>
-      <c r="C38" s="12"/>
-      <c r="D38" s="12"/>
-      <c r="E38" s="12"/>
-      <c r="F38" s="12"/>
+      <c r="B38" s="18"/>
+      <c r="C38" s="18"/>
+      <c r="D38" s="18"/>
+      <c r="E38" s="18"/>
+      <c r="F38" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="A26:F26"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="A38:F38"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="B18:F18"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="A7:F7"/>
@@ -1479,6 +1461,24 @@
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="B20:F20"/>
+    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="B13:F13"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>

</xml_diff>